<commit_message>
fix: chay Isolation Forest voi master moi
</commit_message>
<xml_diff>
--- a/Tho_Order_Anomaly/outputs/anomaly_summary.xlsx
+++ b/Tho_Order_Anomaly/outputs/anomaly_summary.xlsx
@@ -28,7 +28,7 @@
     <t>Phiên bản</t>
   </si>
   <si>
-    <t>isolation_forest_v2_provisional</t>
+    <t>isolation_forest_v3_20261028</t>
   </si>
   <si>
     <t>Số đơn delivered</t>
@@ -49,7 +49,7 @@
     <t>Nguồn</t>
   </si>
   <si>
-    <t>Chờ nhóm xác nhận bản master và dữ liệu sạch chính thức</t>
+    <t>Master nhóm cập nhật 28/10/2026 và bảng đơn sạch trong processed</t>
   </si>
   <si>
     <t>reason</t>
@@ -229,45 +229,45 @@
     <t>70c5c8376c293342409c02ca6d5e4ff0</t>
   </si>
   <si>
+    <t>8272b63d03f5f79c56e9e4120aec44ef</t>
+  </si>
+  <si>
+    <t>4546caea018ad8c692964e3382debd19</t>
+  </si>
+  <si>
+    <t>Phi_van_chuyen_cao; Ty_le_phi_van_chuyen_cao; Nhieu_san_pham</t>
+  </si>
+  <si>
+    <t>a452fba32eab28a4a62af18eed010c0b</t>
+  </si>
+  <si>
+    <t>8797ab21284e4c29f9b4661f05b52da2</t>
+  </si>
+  <si>
     <t>1b3190b2dfa9d789e1f14c05b647a14a</t>
   </si>
   <si>
     <t>eb21169c3153a2b507fc7e76d561ff14</t>
   </si>
   <si>
-    <t>8272b63d03f5f79c56e9e4120aec44ef</t>
-  </si>
-  <si>
-    <t>4546caea018ad8c692964e3382debd19</t>
-  </si>
-  <si>
-    <t>Phi_van_chuyen_cao; Ty_le_phi_van_chuyen_cao; Nhieu_san_pham</t>
-  </si>
-  <si>
-    <t>a452fba32eab28a4a62af18eed010c0b</t>
-  </si>
-  <si>
-    <t>8797ab21284e4c29f9b4661f05b52da2</t>
-  </si>
-  <si>
     <t>525e11b26fdb7f41471d289897d0f6da</t>
   </si>
   <si>
     <t>452ab8cfe9ab69e589da08845df9cebf</t>
   </si>
   <si>
+    <t>2d7561026d542c8dbd8f0daeadf67a43</t>
+  </si>
+  <si>
+    <t>186a453a38d349c487ccbf472b31fb39</t>
+  </si>
+  <si>
     <t>2fa29503f2ebd9f53deba187160f3202</t>
   </si>
   <si>
     <t>9b1c9c3315e0c6f2ceb5da19d67f1baa</t>
   </si>
   <si>
-    <t>2d7561026d542c8dbd8f0daeadf67a43</t>
-  </si>
-  <si>
-    <t>186a453a38d349c487ccbf472b31fb39</t>
-  </si>
-  <si>
     <t>2ba1366baecad3c3536f27546d129017</t>
   </si>
   <si>
@@ -310,18 +310,18 @@
     <t>8a9b30182d557a7b44a8543c9f2fe931</t>
   </si>
   <si>
+    <t>4fbc8d6f2f4db3e789d5a876fa349b56</t>
+  </si>
+  <si>
+    <t>21323ae87907bc6eeb4987c0381bceb9</t>
+  </si>
+  <si>
     <t>4f39a94d6e474819d898d6df7d394996</t>
   </si>
   <si>
     <t>b0cd6a169aaf7502ca3783e5e7527921</t>
   </si>
   <si>
-    <t>4fbc8d6f2f4db3e789d5a876fa349b56</t>
-  </si>
-  <si>
-    <t>21323ae87907bc6eeb4987c0381bceb9</t>
-  </si>
-  <si>
     <t>031e7d4e559a1bf08e71a419aa998d0a</t>
   </si>
   <si>
@@ -337,18 +337,18 @@
     <t>Gia_tri_san_pham_cao; So_ky_tra_gop_cao; Thoi_gian_giao_hang_dai; Giao_hang_tre_nhieu</t>
   </si>
   <si>
+    <t>71dab1155600756af6de79de92e712e3</t>
+  </si>
+  <si>
+    <t>eae0a83d752b1dd32697e0e7b4221656</t>
+  </si>
+  <si>
     <t>da81fbc27b55e0f3d2813cf2078dc780</t>
   </si>
   <si>
     <t>9770456b4233cdf2363287ca2295650a</t>
   </si>
   <si>
-    <t>71dab1155600756af6de79de92e712e3</t>
-  </si>
-  <si>
-    <t>eae0a83d752b1dd32697e0e7b4221656</t>
-  </si>
-  <si>
     <t>cce224811ba8fea016c049693c3e0402</t>
   </si>
   <si>
@@ -385,24 +385,30 @@
     <t>0c0efcea44dc4ff4f9a2d0afa966e609</t>
   </si>
   <si>
+    <t>29c3b79aace1b72a82b1232bf494e16f</t>
+  </si>
+  <si>
+    <t>6411c4f3a3a713893b2a54533129da94</t>
+  </si>
+  <si>
     <t>103188b1afa4614c023b86344f79727b</t>
   </si>
   <si>
     <t>c7d1c1a9792b4c5b53f6e88807ec88f6</t>
   </si>
   <si>
-    <t>29c3b79aace1b72a82b1232bf494e16f</t>
-  </si>
-  <si>
-    <t>6411c4f3a3a713893b2a54533129da94</t>
-  </si>
-  <si>
     <t>c5f43352377291361dad9a7366ae1c89</t>
   </si>
   <si>
     <t>86746b3b1b8b21f33b2e67c362e37cb5</t>
   </si>
   <si>
+    <t>607a624a0fb32899edc4e3f9c9b24189</t>
+  </si>
+  <si>
+    <t>f236ed5552a1074b20a29af39a5c2bab</t>
+  </si>
+  <si>
     <t>ac403e440819af1853b7fcd7f04de6c4</t>
   </si>
   <si>
@@ -412,10 +418,10 @@
     <t>Ty_le_phi_van_chuyen_cao; Thoi_gian_giao_hang_dai; Giao_hang_tre_nhieu</t>
   </si>
   <si>
-    <t>607a624a0fb32899edc4e3f9c9b24189</t>
-  </si>
-  <si>
-    <t>f236ed5552a1074b20a29af39a5c2bab</t>
+    <t>815b68de0bc7fa6c117e4bcf855734ef</t>
+  </si>
+  <si>
+    <t>13f6497d6db06969e7c7a10c914e1a6f</t>
   </si>
   <si>
     <t>af822dacd6f5cff7376413c03a388bb7</t>
@@ -433,12 +439,6 @@
     <t>Gia_tri_san_pham_cao; Phi_van_chuyen_cao; Ty_le_phi_van_chuyen_cao; Nhieu_san_pham</t>
   </si>
   <si>
-    <t>815b68de0bc7fa6c117e4bcf855734ef</t>
-  </si>
-  <si>
-    <t>13f6497d6db06969e7c7a10c914e1a6f</t>
-  </si>
-  <si>
     <t>1e12d5b3e0bc11aa9db357373ccde6f8</t>
   </si>
   <si>
@@ -454,22 +454,25 @@
     <t>232422c2db1f7c69daf3b0f0421ebb43</t>
   </si>
   <si>
+    <t>28f12a3e5117f5e70bbdb45be9188639</t>
+  </si>
+  <si>
+    <t>5d0592e49136297ece57979183c9cac2</t>
+  </si>
+  <si>
     <t>2455cbeb73fd04b170ca2504662f95ce</t>
   </si>
   <si>
     <t>066ee6b9c6fc284260ff9a1274a82ca7</t>
-  </si>
-  <si>
-    <t>28f12a3e5117f5e70bbdb45be9188639</t>
-  </si>
-  <si>
-    <t>5d0592e49136297ece57979183c9cac2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.00%"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -513,9 +516,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -861,7 +865,7 @@
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="2">
         <v>0.01000228031261013</v>
       </c>
     </row>
@@ -870,7 +874,7 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>0.7970204841713222</v>
+        <v>0.7953488372093023</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -916,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="B3">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -924,7 +928,7 @@
         <v>15</v>
       </c>
       <c r="B4">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -932,7 +936,7 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -940,7 +944,7 @@
         <v>17</v>
       </c>
       <c r="B6">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -948,7 +952,7 @@
         <v>18</v>
       </c>
       <c r="B7">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -956,7 +960,7 @@
         <v>19</v>
       </c>
       <c r="B8">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -964,7 +968,7 @@
         <v>20</v>
       </c>
       <c r="B9">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -972,7 +976,7 @@
         <v>21</v>
       </c>
       <c r="B10">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1012,10 +1016,10 @@
         <v>85.90000000000001</v>
       </c>
       <c r="C2">
-        <v>149.4</v>
+        <v>158</v>
       </c>
       <c r="D2">
-        <v>1.7392</v>
+        <v>1.8393</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1026,10 +1030,10 @@
         <v>17.12</v>
       </c>
       <c r="C3">
-        <v>49.5</v>
+        <v>49.68</v>
       </c>
       <c r="D3">
-        <v>2.8914</v>
+        <v>2.9019</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1040,10 +1044,10 @@
         <v>0.2244</v>
       </c>
       <c r="C4">
-        <v>0.3222</v>
+        <v>0.322</v>
       </c>
       <c r="D4">
-        <v>1.4358</v>
+        <v>1.4349</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1093,13 +1097,13 @@
         <v>32</v>
       </c>
       <c r="B8">
-        <v>10.2276</v>
+        <v>10.2274</v>
       </c>
       <c r="C8">
-        <v>25.152</v>
+        <v>25.1996</v>
       </c>
       <c r="D8">
-        <v>2.4592</v>
+        <v>2.4639</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1170,7 +1174,7 @@
         <v>161.7753</v>
       </c>
       <c r="F2">
-        <v>0.2192663820540662</v>
+        <v>0.2193659351082864</v>
       </c>
       <c r="G2" t="s">
         <v>41</v>
@@ -1193,7 +1197,7 @@
         <v>155.6064</v>
       </c>
       <c r="F3">
-        <v>0.2137441162108981</v>
+        <v>0.2147574723345914</v>
       </c>
       <c r="G3" t="s">
         <v>44</v>
@@ -1216,7 +1220,7 @@
         <v>155.4561</v>
       </c>
       <c r="F4">
-        <v>0.2079142376206493</v>
+        <v>0.2074690905217802</v>
       </c>
       <c r="G4" t="s">
         <v>47</v>
@@ -1239,7 +1243,7 @@
         <v>144.6868</v>
       </c>
       <c r="F5">
-        <v>0.2056696025857828</v>
+        <v>0.2057241732648176</v>
       </c>
       <c r="G5" t="s">
         <v>47</v>
@@ -1262,7 +1266,7 @@
         <v>166.5834</v>
       </c>
       <c r="F6">
-        <v>0.2048142913031516</v>
+        <v>0.2053668670253593</v>
       </c>
       <c r="G6" t="s">
         <v>52</v>
@@ -1285,7 +1289,7 @@
         <v>175.8691</v>
       </c>
       <c r="F7">
-        <v>0.2034087696014977</v>
+        <v>0.2031321359100912</v>
       </c>
       <c r="G7" t="s">
         <v>47</v>
@@ -1308,7 +1312,7 @@
         <v>181.6088</v>
       </c>
       <c r="F8">
-        <v>0.1995183191977039</v>
+        <v>0.1987584913444523</v>
       </c>
       <c r="G8" t="s">
         <v>47</v>
@@ -1331,7 +1335,7 @@
         <v>165.6339</v>
       </c>
       <c r="F9">
-        <v>0.19735567563662</v>
+        <v>0.1977389383419339</v>
       </c>
       <c r="G9" t="s">
         <v>47</v>
@@ -1354,7 +1358,7 @@
         <v>161.61</v>
       </c>
       <c r="F10">
-        <v>0.1969558106791782</v>
+        <v>0.1973388978134023</v>
       </c>
       <c r="G10" t="s">
         <v>47</v>
@@ -1377,7 +1381,7 @@
         <v>162.7183</v>
       </c>
       <c r="F11">
-        <v>0.1969097447547209</v>
+        <v>0.1968001213876468</v>
       </c>
       <c r="G11" t="s">
         <v>47</v>
@@ -1400,7 +1404,7 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>0.194367464315095</v>
+        <v>0.1950769386878593</v>
       </c>
       <c r="G12" t="s">
         <v>65</v>
@@ -1423,7 +1427,7 @@
         <v>167.7084</v>
       </c>
       <c r="F13">
-        <v>0.1933744767116312</v>
+        <v>0.1931167634846695</v>
       </c>
       <c r="G13" t="s">
         <v>47</v>
@@ -1446,7 +1450,7 @@
         <v>153.7592</v>
       </c>
       <c r="F14">
-        <v>0.1922204238811636</v>
+        <v>0.1907685286931316</v>
       </c>
       <c r="G14" t="s">
         <v>47</v>
@@ -1463,39 +1467,39 @@
         <v>1</v>
       </c>
       <c r="D15">
-        <v>208.3518</v>
+        <v>14.9886</v>
       </c>
       <c r="E15">
-        <v>188.9751</v>
+        <v>3.7521</v>
       </c>
       <c r="F15">
-        <v>0.1906536954342435</v>
+        <v>0.1904882680670282</v>
       </c>
       <c r="G15" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C16" t="b">
         <v>1</v>
       </c>
       <c r="D16">
-        <v>14.9886</v>
+        <v>167.6015</v>
       </c>
       <c r="E16">
-        <v>3.7521</v>
+        <v>138.5744</v>
       </c>
       <c r="F16">
-        <v>0.1902709246122221</v>
+        <v>0.1899742665081546</v>
       </c>
       <c r="G16" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1509,13 +1513,13 @@
         <v>1</v>
       </c>
       <c r="D17">
-        <v>167.6015</v>
+        <v>208.3518</v>
       </c>
       <c r="E17">
-        <v>138.5744</v>
+        <v>188.9751</v>
       </c>
       <c r="F17">
-        <v>0.1894318230059817</v>
+        <v>0.1899034835918981</v>
       </c>
       <c r="G17" t="s">
         <v>47</v>
@@ -1538,7 +1542,7 @@
         <v>134.6237</v>
       </c>
       <c r="F18">
-        <v>0.188698156713238</v>
+        <v>0.1894363643637775</v>
       </c>
       <c r="G18" t="s">
         <v>47</v>
@@ -1555,13 +1559,13 @@
         <v>1</v>
       </c>
       <c r="D19">
-        <v>172.1395</v>
+        <v>188.1346</v>
       </c>
       <c r="E19">
-        <v>132.7672</v>
+        <v>159.6099</v>
       </c>
       <c r="F19">
-        <v>0.1875522507365198</v>
+        <v>0.1888958348078603</v>
       </c>
       <c r="G19" t="s">
         <v>47</v>
@@ -1578,13 +1582,13 @@
         <v>1</v>
       </c>
       <c r="D20">
-        <v>188.1346</v>
+        <v>172.1395</v>
       </c>
       <c r="E20">
-        <v>159.6099</v>
+        <v>132.7672</v>
       </c>
       <c r="F20">
-        <v>0.1870972380700334</v>
+        <v>0.1872825762057439</v>
       </c>
       <c r="G20" t="s">
         <v>47</v>
@@ -1607,7 +1611,7 @@
         <v>152.6832</v>
       </c>
       <c r="F21">
-        <v>0.1854503172884171</v>
+        <v>0.1853575741225934</v>
       </c>
       <c r="G21" t="s">
         <v>47</v>
@@ -1630,7 +1634,7 @@
         <v>132.6308</v>
       </c>
       <c r="F22">
-        <v>0.1851168491468537</v>
+        <v>0.1850098139159952</v>
       </c>
       <c r="G22" t="s">
         <v>47</v>
@@ -1653,7 +1657,7 @@
         <v>137.63</v>
       </c>
       <c r="F23">
-        <v>0.182585498276517</v>
+        <v>0.1828011546735191</v>
       </c>
       <c r="G23" t="s">
         <v>47</v>
@@ -1676,7 +1680,7 @@
         <v>121.8666</v>
       </c>
       <c r="F24">
-        <v>0.1820037388691975</v>
+        <v>0.1824279622343271</v>
       </c>
       <c r="G24" t="s">
         <v>41</v>
@@ -1699,7 +1703,7 @@
         <v>143.0044</v>
       </c>
       <c r="F25">
-        <v>0.1812914860895663</v>
+        <v>0.1811995745489886</v>
       </c>
       <c r="G25" t="s">
         <v>47</v>
@@ -1722,7 +1726,7 @@
         <v>153.7655</v>
       </c>
       <c r="F26">
-        <v>0.1799239226375648</v>
+        <v>0.1791853500497424</v>
       </c>
       <c r="G26" t="s">
         <v>47</v>
@@ -1745,7 +1749,7 @@
         <v>109.8929</v>
       </c>
       <c r="F27">
-        <v>0.177821965788568</v>
+        <v>0.1761277639105056</v>
       </c>
       <c r="G27" t="s">
         <v>47</v>
@@ -1762,13 +1766,13 @@
         <v>1</v>
       </c>
       <c r="D28">
-        <v>143.8932</v>
+        <v>168.0828</v>
       </c>
       <c r="E28">
-        <v>112.5794</v>
+        <v>134.9846</v>
       </c>
       <c r="F28">
-        <v>0.174659220744245</v>
+        <v>0.1750624943032911</v>
       </c>
       <c r="G28" t="s">
         <v>47</v>
@@ -1785,13 +1789,13 @@
         <v>1</v>
       </c>
       <c r="D29">
-        <v>168.0828</v>
+        <v>143.8932</v>
       </c>
       <c r="E29">
-        <v>134.9846</v>
+        <v>112.5794</v>
       </c>
       <c r="F29">
-        <v>0.1745298665146434</v>
+        <v>0.1742359638482608</v>
       </c>
       <c r="G29" t="s">
         <v>47</v>
@@ -1814,7 +1818,7 @@
         <v>123.6832</v>
       </c>
       <c r="F30">
-        <v>0.1705870073729529</v>
+        <v>0.1725023050552978</v>
       </c>
       <c r="G30" t="s">
         <v>47</v>
@@ -1837,7 +1841,7 @@
         <v>96.70610000000001</v>
       </c>
       <c r="F31">
-        <v>0.1702366516279136</v>
+        <v>0.1718765374173239</v>
       </c>
       <c r="G31" t="s">
         <v>105</v>
@@ -1854,16 +1858,16 @@
         <v>1</v>
       </c>
       <c r="D32">
-        <v>126.1326</v>
+        <v>39.0183</v>
       </c>
       <c r="E32">
-        <v>100.0131</v>
+        <v>0</v>
       </c>
       <c r="F32">
-        <v>0.1681651451392282</v>
+        <v>0.1681423231701153</v>
       </c>
       <c r="G32" t="s">
-        <v>105</v>
+        <v>65</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -1877,16 +1881,16 @@
         <v>1</v>
       </c>
       <c r="D33">
-        <v>39.0183</v>
+        <v>126.1326</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>100.0131</v>
       </c>
       <c r="F33">
-        <v>0.1679298838839868</v>
+        <v>0.1680618302261367</v>
       </c>
       <c r="G33" t="s">
-        <v>65</v>
+        <v>105</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1906,7 +1910,7 @@
         <v>126.6958</v>
       </c>
       <c r="F34">
-        <v>0.1635574892513934</v>
+        <v>0.1628366703557904</v>
       </c>
       <c r="G34" t="s">
         <v>47</v>
@@ -1929,7 +1933,7 @@
         <v>110.977</v>
       </c>
       <c r="F35">
-        <v>0.1611452758897669</v>
+        <v>0.1619361671677355</v>
       </c>
       <c r="G35" t="s">
         <v>47</v>
@@ -1952,7 +1956,7 @@
         <v>119.7587</v>
       </c>
       <c r="F36">
-        <v>0.1608724293495166</v>
+        <v>0.1613960611723808</v>
       </c>
       <c r="G36" t="s">
         <v>47</v>
@@ -1975,7 +1979,7 @@
         <v>80.5821</v>
       </c>
       <c r="F37">
-        <v>0.1575054837041318</v>
+        <v>0.1591173951897956</v>
       </c>
       <c r="G37" t="s">
         <v>105</v>
@@ -1998,7 +2002,7 @@
         <v>104.6652</v>
       </c>
       <c r="F38">
-        <v>0.1571856238643538</v>
+        <v>0.1577068272392162</v>
       </c>
       <c r="G38" t="s">
         <v>47</v>
@@ -2021,7 +2025,7 @@
         <v>104.5682</v>
       </c>
       <c r="F39">
-        <v>0.1561605017386169</v>
+        <v>0.1555942728832248</v>
       </c>
       <c r="G39" t="s">
         <v>47</v>
@@ -2038,13 +2042,13 @@
         <v>1</v>
       </c>
       <c r="D40">
-        <v>118.9696</v>
+        <v>133.2411</v>
       </c>
       <c r="E40">
-        <v>105.5485</v>
+        <v>94.661</v>
       </c>
       <c r="F40">
-        <v>0.1550797513245779</v>
+        <v>0.1554558037412891</v>
       </c>
       <c r="G40" t="s">
         <v>52</v>
@@ -2061,13 +2065,13 @@
         <v>1</v>
       </c>
       <c r="D41">
-        <v>133.2411</v>
+        <v>118.9696</v>
       </c>
       <c r="E41">
-        <v>94.661</v>
+        <v>105.5485</v>
       </c>
       <c r="F41">
-        <v>0.1541615108348624</v>
+        <v>0.1537031134990595</v>
       </c>
       <c r="G41" t="s">
         <v>52</v>
@@ -2090,7 +2094,7 @@
         <v>109.9115</v>
       </c>
       <c r="F42">
-        <v>0.1532803543664407</v>
+        <v>0.1535156838082523</v>
       </c>
       <c r="G42" t="s">
         <v>47</v>
@@ -2107,39 +2111,39 @@
         <v>1</v>
       </c>
       <c r="D43">
-        <v>64.7903</v>
+        <v>124.9978</v>
       </c>
       <c r="E43">
-        <v>37.7966</v>
+        <v>63.4659</v>
       </c>
       <c r="F43">
-        <v>0.1513855036529982</v>
+        <v>0.1510501789857995</v>
       </c>
       <c r="G43" t="s">
-        <v>130</v>
+        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:7">
       <c r="A44" t="s">
+        <v>130</v>
+      </c>
+      <c r="B44" t="s">
         <v>131</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="b">
+        <v>1</v>
+      </c>
+      <c r="D44">
+        <v>64.7903</v>
+      </c>
+      <c r="E44">
+        <v>37.7966</v>
+      </c>
+      <c r="F44">
+        <v>0.1496369941951509</v>
+      </c>
+      <c r="G44" t="s">
         <v>132</v>
-      </c>
-      <c r="C44" t="b">
-        <v>1</v>
-      </c>
-      <c r="D44">
-        <v>124.9978</v>
-      </c>
-      <c r="E44">
-        <v>63.4659</v>
-      </c>
-      <c r="F44">
-        <v>0.1511497596052123</v>
-      </c>
-      <c r="G44" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -2153,16 +2157,16 @@
         <v>1</v>
       </c>
       <c r="D45">
-        <v>10.1823</v>
+        <v>141.9726</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>111.701</v>
       </c>
       <c r="F45">
-        <v>0.1481531850294271</v>
+        <v>0.1482658624324926</v>
       </c>
       <c r="G45" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -2176,39 +2180,39 @@
         <v>1</v>
       </c>
       <c r="D46">
-        <v>13.7728</v>
+        <v>10.1823</v>
       </c>
       <c r="E46">
         <v>0</v>
       </c>
       <c r="F46">
-        <v>0.1475037155091796</v>
+        <v>0.1474406242350823</v>
       </c>
       <c r="G46" t="s">
-        <v>137</v>
+        <v>72</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" t="s">
+        <v>137</v>
+      </c>
+      <c r="B47" t="s">
         <v>138</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="b">
+        <v>1</v>
+      </c>
+      <c r="D47">
+        <v>13.7728</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>0.1470983337963968</v>
+      </c>
+      <c r="G47" t="s">
         <v>139</v>
-      </c>
-      <c r="C47" t="b">
-        <v>1</v>
-      </c>
-      <c r="D47">
-        <v>141.9726</v>
-      </c>
-      <c r="E47">
-        <v>111.701</v>
-      </c>
-      <c r="F47">
-        <v>0.1468936868512987</v>
-      </c>
-      <c r="G47" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -2228,7 +2232,7 @@
         <v>48.9332</v>
       </c>
       <c r="F48">
-        <v>0.146150847357984</v>
+        <v>0.1463587139365449</v>
       </c>
       <c r="G48" t="s">
         <v>142</v>
@@ -2251,7 +2255,7 @@
         <v>106.6953</v>
       </c>
       <c r="F49">
-        <v>0.1448449394712464</v>
+        <v>0.1450523112915084</v>
       </c>
       <c r="G49" t="s">
         <v>47</v>
@@ -2268,16 +2272,16 @@
         <v>1</v>
       </c>
       <c r="D50">
-        <v>10.0011</v>
+        <v>138.8778</v>
       </c>
       <c r="E50">
-        <v>0</v>
+        <v>104.6936</v>
       </c>
       <c r="F50">
-        <v>0.1443401846522611</v>
+        <v>0.143648423687416</v>
       </c>
       <c r="G50" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -2291,16 +2295,16 @@
         <v>1</v>
       </c>
       <c r="D51">
-        <v>138.8778</v>
+        <v>10.0011</v>
       </c>
       <c r="E51">
-        <v>104.6936</v>
+        <v>0</v>
       </c>
       <c r="F51">
-        <v>0.1437463795187568</v>
+        <v>0.1427173716476576</v>
       </c>
       <c r="G51" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>